<commit_message>
docs(safe): align SAFe docs with real codebase (audit findings)
- Fix 20 wrong file references in IMPLEMENTED-BACKLOG.md to match
  actual source files (e.g. gdpr.service.ts → users.controller.ts,
  slack.service.ts → alerting.service.ts, hostname.service.ts →
  hostname.js)
- Fix F-10.1 Leaflet map: ⏳ Backlog → ✅ Done (sites-map.component.ts
  exists with 380 lines, markers, tooltips)
- Fix E-10 status: Partiel → Done
- Fix controller count: 38 → 28 (actual count)
- Fix migration count: 43 → 53
- Fix test counts to reality: 1487→1464 server, 541→554 Angular
- Fix version count: 30+ → 265+
- Update export-to-excel.py test total accordingly

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/safe/NEOPRO_SAFe_Portfolio.xlsx
+++ b/docs/safe/NEOPRO_SAFe_Portfolio.xlsx
@@ -7097,7 +7097,7 @@
       </c>
       <c r="B188" s="4" t="inlineStr">
         <is>
-          <t>2 387</t>
+          <t>2 235</t>
         </is>
       </c>
     </row>
@@ -9215,7 +9215,7 @@
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>2 387</t>
+          <t>2 235</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
@@ -10230,7 +10230,7 @@
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>2 387 tests, coverage</t>
+          <t>2 235 tests, coverage</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">

</xml_diff>

<commit_message>
docs(dual-output): final sync — update all remaining old function references
Update USER-STORIES (US-23.4.4 → resolveDisplayVariant, marked Done),
PROP-011, ADR-031, TROUBLESHOOTING with new function names. Tighten smoke
tests to only accept resolveDisplayVariant (no longer accept old name).
Remove stale agent worktree.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/safe/NEOPRO_SAFe_Portfolio.xlsx
+++ b/docs/safe/NEOPRO_SAFe_Portfolio.xlsx
@@ -11978,18 +11978,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J51"/>
+  <dimension ref="A1:J53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
     <col width="27" customWidth="1" min="2" max="2"/>
-    <col width="49" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
     <col width="46" customWidth="1" min="4" max="4"/>
     <col width="50" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="23" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -13360,11 +13360,11 @@
         <v/>
       </c>
       <c r="F36" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
@@ -13378,17 +13378,17 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>E-17</t>
+          <t>E-15</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>F-17.1</t>
+          <t>F-15.2</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Campagnes A/B Test</t>
+          <t>Lecture directe table de marque multi-constructeurs (Stramatel, Bodet, OCR)</t>
         </is>
       </c>
       <c r="D37" s="4">
@@ -13400,7 +13400,7 @@
         <v/>
       </c>
       <c r="F37" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
@@ -13410,7 +13410,7 @@
       <c r="H37" s="4" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>PI-2 (Avr-Jun 2025)</t>
+          <t>PI-2 (Avr-Mai 2026)</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr"/>
@@ -13418,17 +13418,17 @@
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>E-18</t>
+          <t>E-17</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>F-18.1</t>
+          <t>F-17.1</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Audience réelle via billetterie</t>
+          <t>Campagnes A/B Test</t>
         </is>
       </c>
       <c r="D38" s="4">
@@ -13458,17 +13458,17 @@
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>E-19</t>
+          <t>E-18</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>F-19.1</t>
+          <t>F-18.1</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Comptage spectateurs automatique</t>
+          <t>Audience réelle via billetterie</t>
         </is>
       </c>
       <c r="D39" s="4">
@@ -13480,7 +13480,7 @@
         <v/>
       </c>
       <c r="F39" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
@@ -13498,17 +13498,17 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>E-20</t>
+          <t>E-19</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>F-20.1</t>
+          <t>F-19.1</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Prédictions engagement et uptime</t>
+          <t>Comptage spectateurs automatique</t>
         </is>
       </c>
       <c r="D40" s="4">
@@ -13538,17 +13538,17 @@
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>E-21</t>
+          <t>E-20</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>F-21.1</t>
+          <t>F-20.1</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>API OAuth 2.0 pour partenaires</t>
+          <t>Prédictions engagement et uptime</t>
         </is>
       </c>
       <c r="D41" s="4">
@@ -13578,17 +13578,17 @@
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>E-22</t>
+          <t>E-21</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>F-22.0</t>
+          <t>F-21.1</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Enabler — Validation hardware dual HDMI (spike)</t>
+          <t>API OAuth 2.0 pour partenaires</t>
         </is>
       </c>
       <c r="D42" s="4">
@@ -13600,7 +13600,7 @@
         <v/>
       </c>
       <c r="F42" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
@@ -13610,7 +13610,7 @@
       <c r="H42" s="4" t="inlineStr"/>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>PI-2 (Avr-Jun 2026)</t>
+          <t>PI-2 (Avr-Jun 2025)</t>
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr"/>
@@ -13618,17 +13618,17 @@
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>E-22</t>
+          <t>E-21</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>F-22.1</t>
+          <t>F-21.2</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Dual Kiosk HDMI natif</t>
+          <t>API publique Neopro Live Scores (REST + WebSocket + Webhooks)</t>
         </is>
       </c>
       <c r="D43" s="4">
@@ -13650,7 +13650,7 @@
       <c r="H43" s="4" t="inlineStr"/>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>PI-2 (Avr-Jun 2026)</t>
+          <t>PI-3 (Juin-Juil 2026)</t>
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr"/>
@@ -13663,12 +13663,12 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>F-22.2</t>
+          <t>F-22.0</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Réactions différenciées TV vs LED</t>
+          <t>Enabler — Validation hardware dual HDMI (spike)</t>
         </is>
       </c>
       <c r="D44" s="4">
@@ -13680,7 +13680,7 @@
         <v/>
       </c>
       <c r="F44" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
@@ -13703,12 +13703,12 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>F-22.3</t>
+          <t>F-22.1</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Variantes vidéo par type d'écran</t>
+          <t>Dual Kiosk HDMI natif</t>
         </is>
       </c>
       <c r="D45" s="4">
@@ -13735,103 +13735,183 @@
       </c>
       <c r="J45" s="4" t="inlineStr"/>
     </row>
-    <row r="46"/>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>E-22</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>F-22.2</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>Réactions différenciées TV vs LED</t>
+        </is>
+      </c>
+      <c r="D46" s="4">
+        <f>COUNTIF('User Stories'!B:B,B46)</f>
+        <v/>
+      </c>
+      <c r="E46" s="4">
+        <f>SUMIF('User Stories'!B:B,B46,'User Stories'!E:E)</f>
+        <v/>
+      </c>
+      <c r="F46" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G46" s="4" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="H46" s="4" t="inlineStr"/>
+      <c r="I46" s="4" t="inlineStr">
+        <is>
+          <t>PI-2 (Avr-Jun 2026)</t>
+        </is>
+      </c>
+      <c r="J46" s="4" t="inlineStr"/>
+    </row>
     <row r="47">
-      <c r="A47" s="2" t="inlineStr">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>E-22</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>F-22.3</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>Variantes vidéo par type d'écran</t>
+        </is>
+      </c>
+      <c r="D47" s="4">
+        <f>COUNTIF('User Stories'!B:B,B47)</f>
+        <v/>
+      </c>
+      <c r="E47" s="4">
+        <f>SUMIF('User Stories'!B:B,B47,'User Stories'!E:E)</f>
+        <v/>
+      </c>
+      <c r="F47" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="inlineStr"/>
+      <c r="I47" s="4" t="inlineStr">
+        <is>
+          <t>PI-2 (Avr-Jun 2026)</t>
+        </is>
+      </c>
+      <c r="J47" s="4" t="inlineStr"/>
+    </row>
+    <row r="48"/>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
         <is>
           <t>SUMMARY</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="3" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
         <is>
           <t>PI</t>
         </is>
       </c>
-      <c r="B48" s="3" t="inlineStr">
+      <c r="B50" s="3" t="inlineStr">
         <is>
           <t>Features</t>
         </is>
       </c>
-      <c r="C48" s="3" t="inlineStr">
+      <c r="C50" s="3" t="inlineStr">
         <is>
           <t>Total SP</t>
         </is>
       </c>
-      <c r="D48" s="3" t="inlineStr">
+      <c r="D50" s="3" t="inlineStr">
         <is>
           <t>Terminé</t>
         </is>
       </c>
-      <c r="E48" s="3" t="inlineStr">
+      <c r="E50" s="3" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="4" t="inlineStr">
-        <is>
-          <t>PI-1 (Jan-Mar 2025)</t>
-        </is>
-      </c>
-      <c r="B49" s="4">
-        <f>COUNTIF(I6:I29,"PI-1*")</f>
-        <v/>
-      </c>
-      <c r="C49" s="4">
-        <f>SUMIF(I6:I29,"PI-1*",E6:E29)</f>
-        <v/>
-      </c>
-      <c r="D49" s="4">
-        <f>COUNTIFS(I6:I29,"PI-1*",G6:G29,"Terminé")</f>
-        <v/>
-      </c>
-      <c r="E49" s="4">
-        <f>COUNTIFS(I6:I29,"PI-1*",G6:G29,"Backlog")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="4" t="inlineStr">
-        <is>
-          <t>PI-2 (Avr-Jun 2025)</t>
-        </is>
-      </c>
-      <c r="B50" s="4">
-        <f>COUNTIF(I31:I45,"PI-2*")</f>
-        <v/>
-      </c>
-      <c r="C50" s="4">
-        <f>SUMIF(I31:I45,"PI-2*",E31:E45)</f>
-        <v/>
-      </c>
-      <c r="D50" s="4">
-        <f>COUNTIFS(I31:I45,"PI-2*",G31:G45,"Terminé")</f>
-        <v/>
-      </c>
-      <c r="E50" s="4">
-        <f>COUNTIFS(I31:I45,"PI-2*",G31:G45,"Backlog")</f>
-        <v/>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
+          <t>PI-1 (Jan-Mar 2025)</t>
+        </is>
+      </c>
+      <c r="B51" s="4">
+        <f>COUNTIF(I6:I29,"PI-1*")</f>
+        <v/>
+      </c>
+      <c r="C51" s="4">
+        <f>SUMIF(I6:I29,"PI-1*",E6:E29)</f>
+        <v/>
+      </c>
+      <c r="D51" s="4">
+        <f>COUNTIFS(I6:I29,"PI-1*",G6:G29,"Terminé")</f>
+        <v/>
+      </c>
+      <c r="E51" s="4">
+        <f>COUNTIFS(I6:I29,"PI-1*",G6:G29,"Backlog")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>PI-2 (Avr-Jun 2025)</t>
+        </is>
+      </c>
+      <c r="B52" s="4">
+        <f>COUNTIF(I31:I47,"PI-2*")</f>
+        <v/>
+      </c>
+      <c r="C52" s="4">
+        <f>SUMIF(I31:I47,"PI-2*",E31:E47)</f>
+        <v/>
+      </c>
+      <c r="D52" s="4">
+        <f>COUNTIFS(I31:I47,"PI-2*",G31:G47,"Terminé")</f>
+        <v/>
+      </c>
+      <c r="E52" s="4">
+        <f>COUNTIFS(I31:I47,"PI-2*",G31:G47,"Backlog")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
           <t>PI-3 (Jul-Sep 2025)</t>
         </is>
       </c>
-      <c r="B51" s="4" t="n">
+      <c r="B53" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="C51" s="4" t="n">
+      <c r="C53" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="D51" s="4" t="n">
+      <c r="D53" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E51" s="4" t="n">
+      <c r="E53" s="4" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>